<commit_message>
feat: S3-backed uploads, migration and audit scripts, DB dump/restore helpers
Add private S3 storage with API proxy, migrate-uploads script, and read-key
candidates for legacy layouts. Add audit script for DB upload refs, local DB
dump/restore shell scripts, and dev webpack watch ignores for uploads/logs.
Update DEPLOY.md for Lightsail/RDS. Adjust logger to avoid file logs inside
project cwd during development.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/rating-import-template.xlsx
+++ b/docs/rating-import-template.xlsx
@@ -515,7 +515,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -669,16 +669,130 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TEACHER</v>
+      </c>
+      <c r="B5" t="str">
+        <v>teaching</v>
+      </c>
+      <c r="C5" t="str">
+        <v>教學</v>
+      </c>
+      <c r="D5" t="str">
+        <v>教学</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Teaching</v>
+      </c>
+      <c r="F5" t="str">
+        <v>平淡</v>
+      </c>
+      <c r="G5" t="str">
+        <v>平淡</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Dry</v>
+      </c>
+      <c r="I5" t="str">
+        <v>精彩</v>
+      </c>
+      <c r="J5" t="str">
+        <v>精彩</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Engaging</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TEACHER</v>
+      </c>
+      <c r="B6" t="str">
+        <v>grading</v>
+      </c>
+      <c r="C6" t="str">
+        <v>打分</v>
+      </c>
+      <c r="D6" t="str">
+        <v>给分</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Grading</v>
+      </c>
+      <c r="F6" t="str">
+        <v>嚴苛</v>
+      </c>
+      <c r="G6" t="str">
+        <v>严苛</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Harsh</v>
+      </c>
+      <c r="I6" t="str">
+        <v>友好</v>
+      </c>
+      <c r="J6" t="str">
+        <v>友好</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Generous</v>
+      </c>
+      <c r="L6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TEACHER</v>
+      </c>
+      <c r="B7" t="str">
+        <v>accessibility</v>
+      </c>
+      <c r="C7" t="str">
+        <v>答疑</v>
+      </c>
+      <c r="D7" t="str">
+        <v>答疑</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Accessibility</v>
+      </c>
+      <c r="F7" t="str">
+        <v>難接觸</v>
+      </c>
+      <c r="G7" t="str">
+        <v>难接触</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Hard to reach</v>
+      </c>
+      <c r="I7" t="str">
+        <v>樂於協助</v>
+      </c>
+      <c r="J7" t="str">
+        <v>乐于协助</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Helpful</v>
+      </c>
+      <c r="L7">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -714,26 +828,9 @@
         <v/>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>existing_user_demo</v>
-      </c>
-      <c r="B3" t="str">
-        <v>existing</v>
-      </c>
-      <c r="C3" t="str">
-        <v>replace-with-existing-user-id</v>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>